<commit_message>
Publish the current build
Synced by support/platform/publish_site.py, which checks the site against data/outputs before and after.
</commit_message>
<xml_diff>
--- a/DATA_AUDIT.xlsx
+++ b/DATA_AUDIT.xlsx
@@ -19195,7 +19195,7 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
@@ -19205,14 +19205,22 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>0 found</t>
-        </is>
-      </c>
-      <c r="G213" s="2" t="inlineStr"/>
-      <c r="H213" s="2" t="inlineStr"/>
+          <t>1 found</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>an Excel lockfile among the inputs</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>close the workbook in Excel and re-run</t>
+        </is>
+      </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["~$FINAL_PANEL.xlsx"]</t>
         </is>
       </c>
     </row>

</xml_diff>